<commit_message>
dados: atualização automática 2026-07
</commit_message>
<xml_diff>
--- a/Carga_Energia_ONS_Consolidado.xlsx
+++ b/Carga_Energia_ONS_Consolidado.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Série Histórica" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Apr-2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="May-2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="May-2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Jun-2026" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -249,12 +249,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Série Histórica'!$A$2:$A$62</f>
+              <f>'Série Histórica'!$A$2:$A$61</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Série Histórica'!$F$2:$F$62</f>
+              <f>'Série Histórica'!$F$2:$F$61</f>
             </numRef>
           </val>
         </ser>
@@ -329,7 +329,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>65</row>
+      <row>64</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="5040000"/>
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -684,1253 +684,1233 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>47194.95</v>
+        <v>41136.32</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>16677.27</v>
+        <v>11155.17</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>13779.1</v>
+        <v>12420.57</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>8060.1</v>
+        <v>7981.54</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>85711.42</v>
+        <v>72693.60000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>46114</v>
+        <v>46144</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46997.41</v>
+        <v>40527.29</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>16807.73</v>
+        <v>10849.06</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>13291.52</v>
+        <v>12175.09</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>8007.69</v>
+        <v>8212.219999999999</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>85104.35000000001</v>
+        <v>71763.64999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46115</v>
+        <v>46145</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>41135.67</v>
+        <v>37316.94</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>13356.16</v>
+        <v>8869.860000000001</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>11628.17</v>
+        <v>11889.59</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>7623.48</v>
+        <v>7773.09</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>73743.49000000001</v>
+        <v>65849.48</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>46116</v>
+        <v>46146</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>41945.15</v>
+        <v>42836.93</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>13675.87</v>
+        <v>12608.9</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>12141.36</v>
+        <v>13346.43</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>7907.43</v>
+        <v>8343.68</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>75669.81</v>
+        <v>77135.94</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46117</v>
+        <v>46147</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>40183.07</v>
+        <v>44714.85</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>12245.64</v>
+        <v>13558.25</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>11970.47</v>
+        <v>13529.52</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>7633.39</v>
+        <v>8397.200000000001</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>72032.56</v>
+        <v>80199.81</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>46118</v>
+        <v>46148</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>47858.94</v>
+        <v>45734.72</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>15604.68</v>
+        <v>14481.23</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>13352.92</v>
+        <v>14087.85</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>8290.639999999999</v>
+        <v>8449.610000000001</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>85107.17</v>
+        <v>82753.39999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46119</v>
+        <v>46149</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>49424.79</v>
+        <v>47010.61</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>16286.8</v>
+        <v>14604.03</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>13467.03</v>
+        <v>13716.6</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>8224.309999999999</v>
+        <v>8490.360000000001</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>87402.92999999999</v>
+        <v>83821.61</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>46120</v>
+        <v>46150</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>49506.23</v>
+        <v>47489.39</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>15384.3</v>
+        <v>14025.42</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>13798.61</v>
+        <v>13757.96</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>8431.76</v>
+        <v>8518.24</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>87120.89</v>
+        <v>83791.00999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46121</v>
+        <v>46151</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>49174.08</v>
+        <v>43967.96</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>14789.16</v>
+        <v>11680.14</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>13997.76</v>
+        <v>12827.07</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>8294.559999999999</v>
+        <v>8206.02</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>86255.57000000001</v>
+        <v>76681.19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>46122</v>
+        <v>46152</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>47037.49</v>
+        <v>38337.39</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>14699.36</v>
+        <v>9458.23</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>13951.69</v>
+        <v>12232.62</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>8474.58</v>
+        <v>7721.65</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>84163.11</v>
+        <v>67749.89</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46123</v>
+        <v>46153</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>41571.77</v>
+        <v>41782.62</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>12877.36</v>
+        <v>12591.96</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>13124.36</v>
+        <v>13195.08</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>8145.85</v>
+        <v>8510.219999999999</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>75719.33</v>
+        <v>76079.87</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>46124</v>
+        <v>46154</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>38278.04</v>
+        <v>41852.9</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>11442.8</v>
+        <v>13207.22</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>12177.29</v>
+        <v>13439.31</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>7730.32</v>
+        <v>8436.209999999999</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>69628.45</v>
+        <v>76935.64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46125</v>
+        <v>46155</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>45051.32</v>
+        <v>42756.21</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>14601.08</v>
+        <v>13377.77</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13360.32</v>
+        <v>13345.97</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>8296.68</v>
+        <v>8028.92</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>81309.41</v>
+        <v>77508.88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>46126</v>
+        <v>46156</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>45681.63</v>
+        <v>44224.16</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>15497.39</v>
+        <v>13620.9</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>13880.68</v>
+        <v>13551.3</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>8256.620000000001</v>
+        <v>8389.51</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>83316.32000000001</v>
+        <v>79785.87</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46127</v>
+        <v>46157</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>45538.64</v>
+        <v>45679.32</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>15621.17</v>
+        <v>14342.05</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>13548.48</v>
+        <v>13351.06</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>8287.23</v>
+        <v>8433.639999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>82995.50999999999</v>
+        <v>81806.06</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>46128</v>
+        <v>46158</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>45652.35</v>
+        <v>42414.71</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>15778.2</v>
+        <v>12468.6</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>13713.81</v>
+        <v>12588.7</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>8412.889999999999</v>
+        <v>8245.25</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>83557.25</v>
+        <v>75717.27</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46129</v>
+        <v>46159</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>46724.32</v>
+        <v>39774.07</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>15973.07</v>
+        <v>11513.5</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>13952.42</v>
+        <v>11781.44</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>8378.82</v>
+        <v>7875.91</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>85028.62</v>
+        <v>70944.91</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>46130</v>
+        <v>46160</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>42939.09</v>
+        <v>45245.67</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>13285.4</v>
+        <v>13722.61</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>13323.76</v>
+        <v>13090.18</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>8063.76</v>
+        <v>8639.25</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>77612.00999999999</v>
+        <v>80697.71000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46131</v>
+        <v>46161</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>39204.68</v>
+        <v>45611.15</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>11585.76</v>
+        <v>14037.99</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>12608.25</v>
+        <v>13285.64</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>7677.4</v>
+        <v>8667.23</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>71076.08</v>
+        <v>81602.00999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>46132</v>
+        <v>46162</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>42746.45</v>
+        <v>44527.51</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>13931.85</v>
+        <v>13737.47</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>13618.5</v>
+        <v>13368.69</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>7963.19</v>
+        <v>8698.870000000001</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>78259.99000000001</v>
+        <v>80332.55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46133</v>
+        <v>46163</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>41132.07</v>
+        <v>43306.63</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>13803.91</v>
+        <v>13717.2</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6395.68</v>
+        <v>13585.34</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>7907.58</v>
+        <v>8532.17</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>69239.25</v>
+        <v>79141.33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>46134</v>
+        <v>46164</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45318.63</v>
+        <v>42784.05</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>15475.57</v>
+        <v>14456.1</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>13645.86</v>
+        <v>13497.08</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>8194.18</v>
+        <v>8415.190000000001</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>82634.24000000001</v>
+        <v>79152.42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46135</v>
+        <v>46165</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>45324.78</v>
+        <v>39736.14</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>15668.08</v>
+        <v>12301.63</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>13782.59</v>
+        <v>12842.93</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>8205.57</v>
+        <v>7924.95</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>82981.02</v>
+        <v>72805.64</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>46136</v>
+        <v>46166</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>45849.13</v>
+        <v>36167.59</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>15378.91</v>
+        <v>10741.88</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>13795.45</v>
+        <v>11827.21</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>8223.43</v>
+        <v>7517.93</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>83246.92</v>
+        <v>66254.61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46137</v>
+        <v>46167</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>42969.17</v>
+        <v>42081.45</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>13398.61</v>
+        <v>13889.59</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>12789.74</v>
+        <v>13198.29</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>7946.85</v>
+        <v>8005.06</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>77104.38</v>
+        <v>77174.39</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>46138</v>
+        <v>46168</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>40278.35</v>
+        <v>43614.08</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>11666.25</v>
+        <v>14168.26</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>12008.82</v>
+        <v>13300.75</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>7656.38</v>
+        <v>8143.12</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>71609.78999999999</v>
+        <v>79226.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46139</v>
+        <v>46169</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>47668.78</v>
+        <v>43955.86</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>13579.18</v>
+        <v>13252.09</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>13594.59</v>
+        <v>13587.07</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>8502.440000000001</v>
+        <v>8278.129999999999</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>83344.98</v>
+        <v>79073.16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>46140</v>
+        <v>46170</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>48102.63</v>
+        <v>42814.17</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>14167.91</v>
+        <v>13370.12</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>13829.94</v>
+        <v>13312.35</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>8678.84</v>
+        <v>8329.93</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>84779.32000000001</v>
+        <v>77826.57000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46141</v>
+        <v>46171</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>48312.47</v>
+        <v>42520.69</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>14626.96</v>
+        <v>13599.33</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>13508.46</v>
+        <v>13334.65</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>8847.33</v>
+        <v>8546.15</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>85295.22</v>
+        <v>78000.82000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>46142</v>
+        <v>46172</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>47042.41</v>
+        <v>39402.84</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>13754.05</v>
+        <v>11429.06</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>13534.64</v>
+        <v>13081.19</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>8715.32</v>
+        <v>8342.34</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>83046.41</v>
+        <v>72255.42</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46143</v>
+        <v>46173</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>41136.32</v>
+        <v>35599.76</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>11155.17</v>
+        <v>9988.24</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>12420.57</v>
+        <v>11933.63</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>7981.54</v>
+        <v>7839.48</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>72693.60000000001</v>
+        <v>65361.12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>46144</v>
+        <v>46174</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>40527.29</v>
+        <v>40837.9</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>10849.06</v>
+        <v>13014.66</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>12175.09</v>
+        <v>13211.45</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>8212.219999999999</v>
+        <v>8209.34</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>71763.64999999999</v>
+        <v>75273.35000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46145</v>
+        <v>46175</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>37316.94</v>
+        <v>41151.79</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>8869.860000000001</v>
+        <v>13517.65</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>11889.59</v>
+        <v>13554.95</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>7773.09</v>
+        <v>7757.34</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>65849.48</v>
+        <v>75981.73</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>46146</v>
+        <v>46176</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>42836.93</v>
+        <v>41136.07</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>12608.9</v>
+        <v>13418.1</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>13346.43</v>
+        <v>13586.5</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>8343.68</v>
+        <v>8062.33</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>77135.94</v>
+        <v>76203</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46147</v>
+        <v>46177</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>44714.85</v>
+        <v>38192.11</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>13558.25</v>
+        <v>12288.68</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>13529.52</v>
+        <v>12725.91</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>8397.200000000001</v>
+        <v>7924.08</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>80199.81</v>
+        <v>71130.78</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>46148</v>
+        <v>46178</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>45734.72</v>
+        <v>38780.03</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>14481.23</v>
+        <v>12690.95</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>14087.85</v>
+        <v>12876.81</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>8449.610000000001</v>
+        <v>8475.889999999999</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>82753.39999999999</v>
+        <v>72823.69</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46149</v>
+        <v>46179</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>47010.61</v>
+        <v>36275.89</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>14604.03</v>
+        <v>11315.79</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>13716.6</v>
+        <v>12296.49</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>8490.360000000001</v>
+        <v>7767.14</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>83821.61</v>
+        <v>67655.3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>46150</v>
+        <v>46180</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>47489.39</v>
+        <v>33847</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>14025.42</v>
+        <v>11689.22</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>13757.96</v>
+        <v>11302.29</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>8518.24</v>
+        <v>7920.48</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>83791.00999999999</v>
+        <v>64758.99</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46151</v>
+        <v>46181</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>43967.96</v>
+        <v>39490.15</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>11680.14</v>
+        <v>13880.7</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>12827.07</v>
+        <v>12679.68</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>8206.02</v>
+        <v>8397.42</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>76681.19</v>
+        <v>74447.94</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>46152</v>
+        <v>46182</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>38337.39</v>
+        <v>41321.95</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>9458.23</v>
+        <v>14350.47</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>12232.62</v>
+        <v>12967.63</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>7721.65</v>
+        <v>8263.18</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>67749.89</v>
+        <v>76903.23</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46153</v>
+        <v>46183</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>41782.62</v>
+        <v>42034.78</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>12591.96</v>
+        <v>15052.7</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>13195.08</v>
+        <v>12862.65</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>8510.219999999999</v>
+        <v>8683.84</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>76079.87</v>
+        <v>78633.97</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>46154</v>
+        <v>46184</v>
       </c>
       <c r="B43" s="5" t="n">
-        <v>41852.9</v>
+        <v>43137.91</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>13207.22</v>
+        <v>14704.48</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>13439.31</v>
+        <v>12960.62</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>8436.209999999999</v>
+        <v>8766.48</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>76935.64</v>
+        <v>79569.49000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46155</v>
+        <v>46185</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>42756.21</v>
+        <v>43801.67</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>13377.77</v>
+        <v>14334.18</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>13345.97</v>
+        <v>13176.52</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>8028.92</v>
+        <v>8954.32</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>77508.88</v>
+        <v>80266.67999999999</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>46156</v>
+        <v>46186</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>44224.16</v>
+        <v>41318.53</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>13620.9</v>
+        <v>11823.01</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>13551.3</v>
+        <v>12665.91</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>8389.51</v>
+        <v>8536.5</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>79785.87</v>
+        <v>74343.96000000001</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46157</v>
+        <v>46187</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>45679.32</v>
+        <v>38546.45</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>14342.05</v>
+        <v>10802.42</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>13351.06</v>
+        <v>11862.62</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>8433.639999999999</v>
+        <v>8319.959999999999</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>81806.06</v>
+        <v>69531.46000000001</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>46158</v>
+        <v>46188</v>
       </c>
       <c r="B47" s="5" t="n">
-        <v>42414.71</v>
+        <v>43737.12</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>12468.6</v>
+        <v>14303.99</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>12588.7</v>
+        <v>13181.38</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>8245.25</v>
+        <v>8770.1</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>75717.27</v>
+        <v>79992.59</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46159</v>
+        <v>46189</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>39774.07</v>
+        <v>43822.36</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>11513.5</v>
+        <v>14495.01</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>11781.44</v>
+        <v>13511.63</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>7875.91</v>
+        <v>9028.58</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>70944.91</v>
+        <v>80857.58</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
-        <v>46160</v>
+        <v>46190</v>
       </c>
       <c r="B49" s="5" t="n">
-        <v>45245.67</v>
+        <v>42463.61</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>13722.61</v>
+        <v>14090.62</v>
       </c>
       <c r="D49" s="5" t="n">
-        <v>13090.18</v>
+        <v>13726.15</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>8639.25</v>
+        <v>8662.290000000001</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>80697.71000000001</v>
+        <v>78942.67</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46161</v>
+        <v>46191</v>
       </c>
       <c r="B50" s="3" t="n">
-        <v>45611.15</v>
+        <v>40913.25</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>14037.99</v>
+        <v>14216.3</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>13285.64</v>
+        <v>13630.79</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>8667.23</v>
+        <v>8632.610000000001</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>81602.00999999999</v>
+        <v>77392.94</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>46162</v>
+        <v>46192</v>
       </c>
       <c r="B51" s="5" t="n">
-        <v>44527.51</v>
+        <v>40760.26</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>13737.47</v>
+        <v>14540.79</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>13368.69</v>
+        <v>13302.51</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>8698.870000000001</v>
+        <v>8669.719999999999</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>80332.55</v>
+        <v>77273.28</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46163</v>
+        <v>46193</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>43306.63</v>
+        <v>39113.52</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>13717.2</v>
+        <v>12604.03</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>13585.34</v>
+        <v>12663.12</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>8532.17</v>
+        <v>8522.26</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>79141.33</v>
+        <v>72902.92999999999</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
-        <v>46164</v>
+        <v>46194</v>
       </c>
       <c r="B53" s="5" t="n">
-        <v>42784.05</v>
+        <v>35114.62</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>14456.1</v>
+        <v>10649.44</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>13497.08</v>
+        <v>11755.67</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>8415.190000000001</v>
+        <v>8154.22</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>79152.42</v>
+        <v>65673.94</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46165</v>
+        <v>46195</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>39736.14</v>
+        <v>41019.6</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>12301.63</v>
+        <v>14363.05</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>12842.93</v>
+        <v>13091.48</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>7924.95</v>
+        <v>8598.02</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>72805.64</v>
+        <v>77072.14999999999</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
-        <v>46166</v>
+        <v>46196</v>
       </c>
       <c r="B55" s="5" t="n">
-        <v>36167.59</v>
+        <v>43709.71</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>10741.88</v>
+        <v>14452.46</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>11827.21</v>
+        <v>12910.17</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>7517.93</v>
+        <v>8764.889999999999</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>66254.61</v>
+        <v>79837.24000000001</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46167</v>
+        <v>46197</v>
       </c>
       <c r="B56" s="3" t="n">
-        <v>42081.45</v>
+        <v>43937.15</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>13889.59</v>
+        <v>14394.46</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>13198.29</v>
+        <v>12293.92</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>8005.06</v>
+        <v>8627.889999999999</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>77174.39</v>
+        <v>79253.42</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
-        <v>46168</v>
+        <v>46198</v>
       </c>
       <c r="B57" s="5" t="n">
-        <v>43614.08</v>
+        <v>43879.88</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>14168.26</v>
+        <v>14518.64</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>13300.75</v>
+        <v>13417.04</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>8143.12</v>
+        <v>8403.49</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>79226.2</v>
+        <v>80219.05</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46169</v>
+        <v>46199</v>
       </c>
       <c r="B58" s="3" t="n">
-        <v>43955.86</v>
+        <v>43765.89</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>13252.09</v>
+        <v>14330.93</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>13587.07</v>
+        <v>13536.81</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>8278.129999999999</v>
+        <v>8714.139999999999</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>79073.16</v>
+        <v>80347.78</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
-        <v>46170</v>
+        <v>46200</v>
       </c>
       <c r="B59" s="5" t="n">
-        <v>42814.17</v>
+        <v>40006.48</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>13370.12</v>
+        <v>12699.45</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>13312.35</v>
+        <v>13116.74</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>8329.93</v>
+        <v>8412.969999999999</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>77826.57000000001</v>
+        <v>74235.63</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46171</v>
+        <v>46201</v>
       </c>
       <c r="B60" s="3" t="n">
-        <v>42520.69</v>
+        <v>35867.83</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>13599.33</v>
+        <v>10710.62</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>13334.65</v>
+        <v>11612.13</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>8546.15</v>
+        <v>8097.55</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>78000.82000000001</v>
+        <v>66288.14</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
-        <v>46172</v>
+        <v>46202</v>
       </c>
       <c r="B61" s="5" t="n">
-        <v>39402.84</v>
+        <v>39671.33</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>11429.06</v>
+        <v>12858.11</v>
       </c>
       <c r="D61" s="5" t="n">
-        <v>13081.19</v>
+        <v>12262.33</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>8342.34</v>
+        <v>8376.690000000001</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>72255.42</v>
+        <v>73168.47</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B62" s="3" t="n">
-        <v>35599.76</v>
-      </c>
-      <c r="C62" s="3" t="n">
-        <v>9988.24</v>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>11933.63</v>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>7839.48</v>
-      </c>
-      <c r="F62" s="3" t="n">
-        <v>65361.12</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>MÉDIA DO MÊS</t>
         </is>
       </c>
-      <c r="B63" s="7">
-        <f>AVERAGE(B2:B62)</f>
+      <c r="B62" s="7">
+        <f>AVERAGE(B2:B61)</f>
         <v/>
       </c>
-      <c r="C63" s="7">
-        <f>AVERAGE(C2:C62)</f>
+      <c r="C62" s="7">
+        <f>AVERAGE(C2:C61)</f>
         <v/>
       </c>
-      <c r="D63" s="7">
-        <f>AVERAGE(D2:D62)</f>
+      <c r="D62" s="7">
+        <f>AVERAGE(D2:D61)</f>
         <v/>
       </c>
-      <c r="E63" s="7">
-        <f>AVERAGE(E2:E62)</f>
+      <c r="E62" s="7">
+        <f>AVERAGE(E2:E61)</f>
         <v/>
       </c>
-      <c r="F63" s="7">
-        <f>AVERAGE(F2:F62)</f>
+      <c r="F62" s="7">
+        <f>AVERAGE(F2:F61)</f>
         <v/>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Fonte: ONS – Boletim Diário da Operação (sdro.ons.org.br)</t>
         </is>
@@ -1938,7 +1918,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A64:F64"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1946,697 +1926,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Sudeste/Centro-Oeste</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Sul</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Nordeste</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Norte</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sistema Interligado Nacional</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46113</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>47194.95</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>16677.27</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>13779.1</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>8060.1</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>85711.42</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
-        <v>46114</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>46997.41</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>16807.73</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>13291.52</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>8007.69</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>85104.35000000001</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46115</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>41135.67</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>13356.16</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>11628.17</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>7623.48</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>73743.49000000001</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>46116</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>41945.15</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>13675.87</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>12141.36</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>7907.43</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>75669.81</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>46117</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>40183.07</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>12245.64</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>11970.47</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>7633.39</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>72032.56</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>46118</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>47858.94</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>15604.68</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>13352.92</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>8290.639999999999</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>85107.17</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46119</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>49424.79</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>16286.8</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>13467.03</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>8224.309999999999</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>87402.92999999999</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>46120</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>49506.23</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>15384.3</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>13798.61</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>8431.76</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>87120.89</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46121</v>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>49174.08</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>14789.16</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>13997.76</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>8294.559999999999</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>86255.57000000001</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>47037.49</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>14699.36</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>13951.69</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>8474.58</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>84163.11</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>41571.77</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>12877.36</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>13124.36</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>8145.85</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>75719.33</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>38278.04</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>11442.8</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>12177.29</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>7730.32</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>69628.45</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>45051.32</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>14601.08</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>13360.32</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>8296.68</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>81309.41</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>46126</v>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>45681.63</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>15497.39</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>13880.68</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>8256.620000000001</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>83316.32000000001</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46127</v>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>45538.64</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>15621.17</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>13548.48</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>8287.23</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>82995.50999999999</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>45652.35</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>15778.2</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>13713.81</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>8412.889999999999</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>83557.25</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46129</v>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>46724.32</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>15973.07</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>13952.42</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>8378.82</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>85028.62</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>42939.09</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>13285.4</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>13323.76</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>8063.76</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>77612.00999999999</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46131</v>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>39204.68</v>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>11585.76</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>12608.25</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>7677.4</v>
-      </c>
-      <c r="F20" s="3" t="n">
-        <v>71076.08</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>46132</v>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>42746.45</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>13931.85</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>13618.5</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>7963.19</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>78259.99000000001</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>41132.07</v>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>13803.91</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>6395.68</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>7907.58</v>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>69239.25</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>46134</v>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>45318.63</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>15475.57</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>13645.86</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>8194.18</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>82634.24000000001</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>46135</v>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>45324.78</v>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>15668.08</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>13782.59</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>8205.57</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>82981.02</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>45849.13</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>15378.91</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>13795.45</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>8223.43</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>83246.92</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B26" s="3" t="n">
-        <v>42969.17</v>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>13398.61</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>12789.74</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>7946.85</v>
-      </c>
-      <c r="F26" s="3" t="n">
-        <v>77104.38</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>46138</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>40278.35</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>11666.25</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>12008.82</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>7656.38</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>71609.78999999999</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>46139</v>
-      </c>
-      <c r="B28" s="3" t="n">
-        <v>47668.78</v>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>13579.18</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>13594.59</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>8502.440000000001</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>83344.98</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>46140</v>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>48102.63</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>14167.91</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>13829.94</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>8678.84</v>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>84779.32000000001</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>46141</v>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>48312.47</v>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>14626.96</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>13508.46</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>8847.33</v>
-      </c>
-      <c r="F30" s="3" t="n">
-        <v>85295.22</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>47042.41</v>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>13754.05</v>
-      </c>
-      <c r="D31" s="5" t="n">
-        <v>13534.64</v>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>8715.32</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>83046.41</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>MÉDIA DO MÊS</t>
-        </is>
-      </c>
-      <c r="B32" s="7">
-        <f>AVERAGE(B2:B31)</f>
-        <v/>
-      </c>
-      <c r="C32" s="7">
-        <f>AVERAGE(C2:C31)</f>
-        <v/>
-      </c>
-      <c r="D32" s="7">
-        <f>AVERAGE(D2:D31)</f>
-        <v/>
-      </c>
-      <c r="E32" s="7">
-        <f>AVERAGE(E2:E31)</f>
-        <v/>
-      </c>
-      <c r="F32" s="7">
-        <f>AVERAGE(F2:F31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>Fonte: ONS – Boletim Diário da Operação (sdro.ons.org.br)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A34:F34"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3345,4 +2634,675 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Sistema Interligado Nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>40837.9</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>13014.66</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13211.45</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>8209.34</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>75273.35000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>41151.79</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>13517.65</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>13554.95</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>7757.34</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>75981.73</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>41136.07</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>13418.1</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>13586.5</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>8062.33</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>76203</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>38192.11</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>12288.68</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>12725.91</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>7924.08</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>71130.78</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>38780.03</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>12690.95</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>12876.81</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>8475.889999999999</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>72823.69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>36275.89</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>11315.79</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>12296.49</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>7767.14</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>67655.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>33847</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>11689.22</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>11302.29</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>7920.48</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>64758.99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>39490.15</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>13880.7</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>12679.68</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>8397.42</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>74447.94</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>41321.95</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>14350.47</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>12967.63</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>8263.18</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>76903.23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>42034.78</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>15052.7</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>12862.65</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>8683.84</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>78633.97</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>43137.91</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>14704.48</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>12960.62</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>8766.48</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>79569.49000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>43801.67</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>14334.18</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>13176.52</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>8954.32</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>80266.67999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>41318.53</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>11823.01</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>12665.91</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>8536.5</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>74343.96000000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>38546.45</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>10802.42</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>11862.62</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>8319.959999999999</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>69531.46000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>43737.12</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>14303.99</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>13181.38</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>8770.1</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>79992.59</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>43822.36</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>14495.01</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>13511.63</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>9028.58</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>80857.58</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>42463.61</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>14090.62</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>13726.15</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>8662.290000000001</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>78942.67</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>40913.25</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>14216.3</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>13630.79</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>8632.610000000001</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>77392.94</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>40760.26</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>14540.79</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>13302.51</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>8669.719999999999</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>77273.28</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>39113.52</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>12604.03</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>12663.12</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>8522.26</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>72902.92999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>35114.62</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>10649.44</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>11755.67</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>8154.22</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>65673.94</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>41019.6</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>14363.05</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>13091.48</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>8598.02</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>77072.14999999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>43709.71</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>14452.46</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>12910.17</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>8764.889999999999</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>79837.24000000001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>43937.15</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>14394.46</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>12293.92</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>8627.889999999999</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>79253.42</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>43879.88</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>14518.64</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>13417.04</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>8403.49</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>80219.05</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>43765.89</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>14330.93</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>13536.81</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>8714.139999999999</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>80347.78</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>40006.48</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>12699.45</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>13116.74</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>8412.969999999999</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>74235.63</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>35867.83</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>10710.62</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>11612.13</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>8097.55</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>66288.14</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>39671.33</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>12858.11</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>12262.33</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>8376.690000000001</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>73168.47</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>MÉDIA DO MÊS</t>
+        </is>
+      </c>
+      <c r="B31" s="7">
+        <f>AVERAGE(B2:B30)</f>
+        <v/>
+      </c>
+      <c r="C31" s="7">
+        <f>AVERAGE(C2:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="7">
+        <f>AVERAGE(D2:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="7">
+        <f>AVERAGE(E2:E30)</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>AVERAGE(F2:F30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Fonte: ONS – Boletim Diário da Operação (sdro.ons.org.br)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A33:F33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>